<commit_message>
Generate latest stock screener reports
</commit_message>
<xml_diff>
--- a/output/debt_free_blue_chip.xlsx
+++ b/output/debt_free_blue_chip.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG19"/>
+  <dimension ref="A1:AG17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -597,7 +597,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -716,7 +716,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -835,7 +835,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -954,7 +954,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>677</v>
+        <v>674</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1188,7 +1188,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1303,7 +1303,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>675</v>
+        <v>672</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1656,7 +1656,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1892,7 +1892,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>982</v>
+        <v>964</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -2479,242 +2479,6 @@
       </c>
       <c r="AG17" t="n">
         <v>29.91292783377705</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>886</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>SIEMENS</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>7.26056043496445</v>
-      </c>
-      <c r="E18" t="n">
-        <v>9.795064826432455</v>
-      </c>
-      <c r="F18" t="n">
-        <v>22.74633123689727</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>56.53846153846154</v>
-      </c>
-      <c r="I18" t="n">
-        <v>1.17690490253987</v>
-      </c>
-      <c r="J18" t="n">
-        <v>267</v>
-      </c>
-      <c r="K18" t="n">
-        <v>264</v>
-      </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="n">
-        <v>56.11764705882353</v>
-      </c>
-      <c r="N18" t="n">
-        <v>24</v>
-      </c>
-      <c r="O18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>https://mkt.in/static/mkt-icons/nifty100/SIEMENS.png</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>Siemens Ltd</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>https://in.tradingview.com/chart/qGsydD2w/?symbol=NSE%3AAMBUJACEM.T0</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>Siemens Limited offers products, integrated solutions for industrial applications for manufacturing industries, drives for process</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>https://www.siemens.com/in/en.html</t>
-        </is>
-      </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>https://www.nseindia.com/get-quotes/equity?symbol=SIEMENS</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>https://www.bseindia.com/stock-share-price/siemens-ltd/SIEMENS/500550/</t>
-        </is>
-      </c>
-      <c r="X18" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>431</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>25.6</v>
-      </c>
-      <c r="AA18" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="AB18" t="n">
-        <v>10.8933932408866</v>
-      </c>
-      <c r="AC18" t="n">
-        <v>42.75412607818098</v>
-      </c>
-      <c r="AD18" t="n">
-        <v>2.836201402166985</v>
-      </c>
-      <c r="AE18" t="n">
-        <v>4.755551956343865</v>
-      </c>
-      <c r="AF18" t="n">
-        <v>100</v>
-      </c>
-      <c r="AG18" t="n">
-        <v>28.40630832601429</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>887</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>SIEMENS</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>5.647124929762128</v>
-      </c>
-      <c r="E19" t="n">
-        <v>1.114440906536805</v>
-      </c>
-      <c r="F19" t="n">
-        <v>13.78285714285714</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
-        <v>35.61290322580645</v>
-      </c>
-      <c r="I19" t="n">
-        <v>1.037706511175899</v>
-      </c>
-      <c r="J19" t="n">
-        <v>738</v>
-      </c>
-      <c r="K19" t="n">
-        <v>130</v>
-      </c>
-      <c r="L19" t="n">
-        <v>17</v>
-      </c>
-      <c r="M19" t="n">
-        <v>61.61971830985915</v>
-      </c>
-      <c r="N19" t="n">
-        <v>35</v>
-      </c>
-      <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="n">
-        <v>608</v>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>https://mkt.in/static/mkt-icons/nifty100/SIEMENS.png</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>Siemens Ltd</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>https://in.tradingview.com/chart/qGsydD2w/?symbol=NSE%3AAMBUJACEM.T0</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>Siemens Limited offers products, integrated solutions for industrial applications for manufacturing industries, drives for process</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>https://www.siemens.com/in/en.html</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>https://www.nseindia.com/get-quotes/equity?symbol=SIEMENS</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>https://www.bseindia.com/stock-share-price/siemens-ltd/SIEMENS/500550/</t>
-        </is>
-      </c>
-      <c r="X19" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>431</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>25.6</v>
-      </c>
-      <c r="AA19" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="AB19" t="n">
-        <v>6.600716452970541</v>
-      </c>
-      <c r="AC19" t="n">
-        <v>33.2533408941277</v>
-      </c>
-      <c r="AD19" t="n">
-        <v>7.839388145315487</v>
-      </c>
-      <c r="AE19" t="n">
-        <v>4.193089194108557</v>
-      </c>
-      <c r="AF19" t="n">
-        <v>100</v>
-      </c>
-      <c r="AG19" t="n">
-        <v>25.94810548583918</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completed stock screener engine and generated screener reports
</commit_message>
<xml_diff>
--- a/output/debt_free_blue_chip.xlsx
+++ b/output/debt_free_blue_chip.xlsx
@@ -425,171 +425,236 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG17"/>
+  <dimension ref="A1:AT17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>id_x</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>company_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>net_profit_margin_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>operating_profit_margin_pct</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>return_on_equity_pct</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>debt_to_equity</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>interest_coverage</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>asset_turnover</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>free_cash_flow_cr</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>capex_cr</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>earnings_per_share</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>book_value_per_share</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>dividend_payout_ratio_pct</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>total_debt_cr</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>cash_from_operations_cr</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>company_logo</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>company_name</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>chart_link</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>about_company</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>website</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>nse_profile</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>bse_profile</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>face_value</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>book_value</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>roce_percentage</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>roe_percentage</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>id_y</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>market_cap_crore</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>enterprise_value_crore</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>pe_ratio</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>pb_ratio</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>ev_ebitda</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>dividend_yield_pct</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>company_id</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>net_profit_margin_pct</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>operating_profit_margin_pct</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>return_on_equity_pct</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>debt_to_equity</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>interest_coverage</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>asset_turnover</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>free_cash_flow_cr</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>capex_cr</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>earnings_per_share</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>book_value_per_share</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>dividend_payout_ratio_pct</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>total_debt_cr</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>cash_from_operations_cr</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>company_logo</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>company_name</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>chart_link</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>about_company</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>website</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>nse_profile</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>bse_profile</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>face_value</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>book_value</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>roce_percentage</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>roe_percentage</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>compounded_sales_growth</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>compounded_profit_growth</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>stock_price_cagr</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>roe</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>roe_score</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>npm_score</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>fcf_score</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>asset_score</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>de_score</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>composite_quality_score</t>
         </is>
@@ -604,10 +669,8 @@
           <t>HINDUNILVR</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
+      <c r="C2" t="n">
+        <v>2020</v>
       </c>
       <c r="D2" t="n">
         <v>16.98212804464218</v>
@@ -696,21 +759,50 @@
         <v>20.2</v>
       </c>
       <c r="AB2" t="n">
+        <v>254</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>365239.67</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>374855.61</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>22.92</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>12.11</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="n">
+        <v>39783</v>
+      </c>
+      <c r="AO2" t="n">
         <v>39.31827002603475</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AP2" t="n">
         <v>100</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AQ2" t="n">
         <v>100</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AR2" t="n">
         <v>7.976592095571338</v>
       </c>
-      <c r="AF2" t="n">
+      <c r="AS2" t="n">
         <v>100</v>
       </c>
-      <c r="AG2" t="n">
+      <c r="AT2" t="n">
         <v>69.5590537186693</v>
       </c>
     </row>
@@ -723,10 +815,8 @@
           <t>LT</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
+      <c r="C3" t="n">
+        <v>2017</v>
       </c>
       <c r="D3" t="n">
         <v>5.933474824355972</v>
@@ -814,22 +904,37 @@
       <c r="AA3" t="n">
         <v>10.49</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="n">
+        <v>109312</v>
+      </c>
+      <c r="AO3" t="n">
         <v>98.79756236238511</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AP3" t="n">
         <v>34.9395247094958</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AQ3" t="n">
         <v>-33.36520076481835</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AR3" t="n">
         <v>100</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="AS3" t="n">
         <v>100</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="AT3" t="n">
         <v>59.89401161577027</v>
       </c>
     </row>
@@ -842,10 +947,8 @@
           <t>HINDUNILVR</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
+      <c r="C4" t="n">
+        <v>2018</v>
       </c>
       <c r="D4" t="n">
         <v>14.70530313686876</v>
@@ -933,22 +1036,37 @@
       <c r="AA4" t="n">
         <v>20.2</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="n">
+        <v>35545</v>
+      </c>
+      <c r="AO4" t="n">
         <v>34.38058732025149</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AP4" t="n">
         <v>86.59281745027381</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AQ4" t="n">
         <v>53.06989589972382</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AR4" t="n">
         <v>8.040961680144312</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="AS4" t="n">
         <v>100</v>
       </c>
-      <c r="AG4" t="n">
+      <c r="AT4" t="n">
         <v>55.76984440010198</v>
       </c>
     </row>
@@ -961,10 +1079,8 @@
           <t>LT</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
+      <c r="C5" t="n">
+        <v>2018</v>
       </c>
       <c r="D5" t="n">
         <v>6.687666585897746</v>
@@ -1052,22 +1168,37 @@
       <c r="AA5" t="n">
         <v>10.49</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="n">
+        <v>119683</v>
+      </c>
+      <c r="AO5" t="n">
         <v>99.30511019681209</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AP5" t="n">
         <v>39.38061571740231</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AQ5" t="n">
         <v>-64.97769279796049</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AR5" t="n">
         <v>90.6139000332507</v>
       </c>
-      <c r="AF5" t="n">
+      <c r="AS5" t="n">
         <v>100</v>
       </c>
-      <c r="AG5" t="n">
+      <c r="AT5" t="n">
         <v>53.69876315609767</v>
       </c>
     </row>
@@ -1080,10 +1211,8 @@
           <t>LTIM</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
+      <c r="C6" t="n">
+        <v>2019</v>
       </c>
       <c r="D6" t="n">
         <v>16.04912132119416</v>
@@ -1168,21 +1297,50 @@
         <v>26.04</v>
       </c>
       <c r="AB6" t="n">
+        <v>367</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>1328108.48</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>1702596.39</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>60.16</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="n">
+        <v>9446</v>
+      </c>
+      <c r="AO6" t="n">
         <v>14.83801507291769</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AP6" t="n">
         <v>94.50594930744036</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AQ6" t="n">
         <v>6.862120246441471</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AR6" t="n">
         <v>5.727597775790644</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="AS6" t="n">
         <v>100</v>
       </c>
-      <c r="AG6" t="n">
+      <c r="AT6" t="n">
         <v>41.03967896387663</v>
       </c>
     </row>
@@ -1195,10 +1353,8 @@
           <t>LTIM</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
+      <c r="C7" t="n">
+        <v>2018</v>
       </c>
       <c r="D7" t="n">
         <v>15.22036682179031</v>
@@ -1282,22 +1438,37 @@
       <c r="AA7" t="n">
         <v>26.04</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="n">
+        <v>7306</v>
+      </c>
+      <c r="AO7" t="n">
         <v>13.79651206132622</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AP7" t="n">
         <v>89.62579237289579</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AQ7" t="n">
         <v>4.164011047376248</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AR7" t="n">
         <v>5.531488629487309</v>
       </c>
-      <c r="AF7" t="n">
+      <c r="AS7" t="n">
         <v>100</v>
       </c>
-      <c r="AG7" t="n">
+      <c r="AT7" t="n">
         <v>39.13988876846732</v>
       </c>
     </row>
@@ -1310,10 +1481,8 @@
           <t>LTIM</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
+      <c r="C8" t="n">
+        <v>2017</v>
       </c>
       <c r="D8" t="n">
         <v>14.93616366712813</v>
@@ -1397,22 +1566,37 @@
       <c r="AA8" t="n">
         <v>26.04</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="n">
+        <v>6501</v>
+      </c>
+      <c r="AO8" t="n">
         <v>14.79069273109404</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AP8" t="n">
         <v>87.9522497290347</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AQ8" t="n">
         <v>2.220097726789887</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="AR8" t="n">
         <v>5.947197014051522</v>
       </c>
-      <c r="AF8" t="n">
+      <c r="AS8" t="n">
         <v>100</v>
       </c>
-      <c r="AG8" t="n">
+      <c r="AT8" t="n">
         <v>38.80593164845298</v>
       </c>
     </row>
@@ -1425,10 +1609,8 @@
           <t>ABB</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
+      <c r="C9" t="n">
+        <v>2019</v>
       </c>
       <c r="D9" t="n">
         <v>12.23158466974721</v>
@@ -1517,21 +1699,50 @@
         <v>34.9</v>
       </c>
       <c r="AB9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>844312.98</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>814410.48</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>19.29</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>14.26</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>22.84</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="n">
+        <v>3679</v>
+      </c>
+      <c r="AO9" t="n">
         <v>10.73249334072148</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AP9" t="n">
         <v>72.02621860813402</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AQ9" t="n">
         <v>2.570639473125133</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AR9" t="n">
         <v>5.054687630643085</v>
       </c>
-      <c r="AF9" t="n">
+      <c r="AS9" t="n">
         <v>100</v>
       </c>
-      <c r="AG9" t="n">
+      <c r="AT9" t="n">
         <v>34.18121304856866</v>
       </c>
     </row>
@@ -1544,10 +1755,8 @@
           <t>ABB</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
+      <c r="C10" t="n">
+        <v>2018</v>
       </c>
       <c r="D10" t="n">
         <v>12.15888417222559</v>
@@ -1635,22 +1844,37 @@
       <c r="AA10" t="n">
         <v>34.9</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="n">
+        <v>3298</v>
+      </c>
+      <c r="AO10" t="n">
         <v>11.34329526533526</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AP10" t="n">
         <v>71.59811856477955</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AQ10" t="n">
         <v>-0.6585935840237944</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AR10" t="n">
         <v>5.515860579402345</v>
       </c>
-      <c r="AF10" t="n">
+      <c r="AS10" t="n">
         <v>100</v>
       </c>
-      <c r="AG10" t="n">
+      <c r="AT10" t="n">
         <v>33.70964439695872</v>
       </c>
     </row>
@@ -1663,10 +1887,8 @@
           <t>LT</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
+      <c r="C11" t="n">
+        <v>2019</v>
       </c>
       <c r="D11" t="n">
         <v>7.555834935660405</v>
@@ -1755,21 +1977,50 @@
         <v>10.49</v>
       </c>
       <c r="AB11" t="n">
+        <v>361</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>685872.9300000001</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>876598.39</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>60.92</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>31.09</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="n">
+        <v>135220</v>
+      </c>
+      <c r="AO11" t="n">
         <v>100</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AP11" t="n">
         <v>44.49286282495233</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AQ11" t="n">
         <v>-167.6120671340556</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AR11" t="n">
         <v>81.99087139978943</v>
       </c>
-      <c r="AF11" t="n">
+      <c r="AS11" t="n">
         <v>100</v>
       </c>
-      <c r="AG11" t="n">
+      <c r="AT11" t="n">
         <v>33.57524627815828</v>
       </c>
     </row>
@@ -1782,10 +2033,8 @@
           <t>ABB</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
+      <c r="C12" t="n">
+        <v>2015</v>
       </c>
       <c r="D12" t="n">
         <v>10.00436871996505</v>
@@ -1871,22 +2120,37 @@
       <c r="AA12" t="n">
         <v>34.9</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr"/>
+      <c r="AN12" t="n">
+        <v>2289</v>
+      </c>
+      <c r="AO12" t="n">
         <v>11.70436114751723</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AP12" t="n">
         <v>58.91116056636613</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AQ12" t="n">
         <v>0.2974293605268749</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="AR12" t="n">
         <v>6.731604915348272</v>
       </c>
-      <c r="AF12" t="n">
+      <c r="AS12" t="n">
         <v>100</v>
       </c>
-      <c r="AG12" t="n">
+      <c r="AT12" t="n">
         <v>31.61140487854446</v>
       </c>
     </row>
@@ -1899,10 +2163,8 @@
           <t>TITAN</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2013</t>
-        </is>
+      <c r="C13" t="n">
+        <v>2013</v>
       </c>
       <c r="D13" t="n">
         <v>7.161908525140769</v>
@@ -1990,22 +2252,37 @@
       <c r="AA13" t="n">
         <v>32.9</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="inlineStr"/>
+      <c r="AN13" t="n">
+        <v>10123</v>
+      </c>
+      <c r="AO13" t="n">
         <v>17.62477586624065</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="AP13" t="n">
         <v>42.17321001416152</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AQ13" t="n">
         <v>4.365838113448056</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="AR13" t="n">
         <v>6.951781792593975</v>
       </c>
-      <c r="AF13" t="n">
+      <c r="AS13" t="n">
         <v>100</v>
       </c>
-      <c r="AG13" t="n">
+      <c r="AT13" t="n">
         <v>31.17165935796554</v>
       </c>
     </row>
@@ -2018,10 +2295,8 @@
           <t>ABB</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>2016</t>
-        </is>
+      <c r="C14" t="n">
+        <v>2016</v>
       </c>
       <c r="D14" t="n">
         <v>9.755164498852334</v>
@@ -2109,22 +2384,37 @@
       <c r="AA14" t="n">
         <v>34.9</v>
       </c>
-      <c r="AB14" t="n">
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="inlineStr"/>
+      <c r="AN14" t="n">
+        <v>2614</v>
+      </c>
+      <c r="AO14" t="n">
         <v>10.2193693913213</v>
       </c>
-      <c r="AC14" t="n">
+      <c r="AP14" t="n">
         <v>57.44371066575524</v>
       </c>
-      <c r="AD14" t="n">
+      <c r="AQ14" t="n">
         <v>1.827066071807945</v>
       </c>
-      <c r="AE14" t="n">
+      <c r="AR14" t="n">
         <v>6.53617671897825</v>
       </c>
-      <c r="AF14" t="n">
+      <c r="AS14" t="n">
         <v>100</v>
       </c>
-      <c r="AG14" t="n">
+      <c r="AT14" t="n">
         <v>31.08455230637292</v>
       </c>
     </row>
@@ -2137,10 +2427,8 @@
           <t>ABB</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
+      <c r="C15" t="n">
+        <v>2017</v>
       </c>
       <c r="D15" t="n">
         <v>9.541853255253187</v>
@@ -2228,22 +2516,37 @@
       <c r="AA15" t="n">
         <v>34.9</v>
       </c>
-      <c r="AB15" t="n">
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr"/>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr"/>
+      <c r="AM15" t="inlineStr"/>
+      <c r="AN15" t="n">
+        <v>2903</v>
+      </c>
+      <c r="AO15" t="n">
         <v>9.564342731719524</v>
       </c>
-      <c r="AC15" t="n">
+      <c r="AP15" t="n">
         <v>56.18761812518317</v>
       </c>
-      <c r="AD15" t="n">
+      <c r="AQ15" t="n">
         <v>1.614616528574464</v>
       </c>
-      <c r="AE15" t="n">
+      <c r="AR15" t="n">
         <v>5.6777501517544</v>
       </c>
-      <c r="AF15" t="n">
+      <c r="AS15" t="n">
         <v>100</v>
       </c>
-      <c r="AG15" t="n">
+      <c r="AT15" t="n">
         <v>30.4757419020288</v>
       </c>
     </row>
@@ -2256,10 +2559,8 @@
           <t>ABB</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
+      <c r="C16" t="n">
+        <v>2014</v>
       </c>
       <c r="D16" t="n">
         <v>8.699472759226714</v>
@@ -2345,22 +2646,37 @@
       <c r="AA16" t="n">
         <v>34.9</v>
       </c>
-      <c r="AB16" t="n">
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr"/>
+      <c r="AM16" t="inlineStr"/>
+      <c r="AN16" t="n">
+        <v>2276</v>
+      </c>
+      <c r="AO16" t="n">
         <v>12.03346766039879</v>
       </c>
-      <c r="AC16" t="n">
+      <c r="AP16" t="n">
         <v>51.22722391656546</v>
       </c>
-      <c r="AD16" t="n">
+      <c r="AQ16" t="n">
         <v>0.1168472487784151</v>
       </c>
-      <c r="AE16" t="n">
+      <c r="AR16" t="n">
         <v>8.07435969861397</v>
       </c>
-      <c r="AF16" t="n">
+      <c r="AS16" t="n">
         <v>100</v>
       </c>
-      <c r="AG16" t="n">
+      <c r="AT16" t="n">
         <v>30.28796388406975</v>
       </c>
     </row>
@@ -2373,10 +2689,8 @@
           <t>ABB</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
+      <c r="C17" t="n">
+        <v>2012</v>
       </c>
       <c r="D17" t="n">
         <v>8.771929824561402</v>
@@ -2462,22 +2776,37 @@
       <c r="AA17" t="n">
         <v>34.9</v>
       </c>
-      <c r="AB17" t="n">
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr"/>
+      <c r="AM17" t="inlineStr"/>
+      <c r="AN17" t="n">
+        <v>1653</v>
+      </c>
+      <c r="AO17" t="n">
         <v>10.73286196491316</v>
       </c>
-      <c r="AC17" t="n">
+      <c r="AP17" t="n">
         <v>51.65389049889376</v>
       </c>
-      <c r="AD17" t="n">
+      <c r="AQ17" t="n">
         <v>0.4461440407903123</v>
       </c>
-      <c r="AE17" t="n">
+      <c r="AR17" t="n">
         <v>7.364192381206283</v>
       </c>
-      <c r="AF17" t="n">
+      <c r="AS17" t="n">
         <v>100</v>
       </c>
-      <c r="AG17" t="n">
+      <c r="AT17" t="n">
         <v>29.91292783377705</v>
       </c>
     </row>

</xml_diff>